<commit_message>
refactor(appium): clarify logout test case descriptions for TC-APP-AUTH-028 and TC-APP-TAB-030
</commit_message>
<xml_diff>
--- a/appium_test_suite/appium_test_analysis_report.xlsx
+++ b/appium_test_suite/appium_test_analysis_report.xlsx
@@ -2208,7 +2208,7 @@
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>Tap Logout button in Tab 1</t>
+          <t>Tap primary header Logout button in Tab 1</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
@@ -16248,7 +16248,7 @@
       </c>
       <c r="E341" s="8" t="inlineStr">
         <is>
-          <t>Tap Logout button in Tab 1 menu</t>
+          <t>Trigger session logout from user avatar dropdown menu in Tab 1</t>
         </is>
       </c>
       <c r="F341" s="12" t="inlineStr">

</xml_diff>